<commit_message>
Added a loader for forecast models and edited Hyper_param_search in SVR folder
</commit_message>
<xml_diff>
--- a/Shallow learners/SVR2/SVM hyper parameter search.xlsx
+++ b/Shallow learners/SVR2/SVM hyper parameter search.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/59168efb92a48cee/Delt skrivebord/Data Science/Speciale/Energinet/Shallow learners/SVM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/59168efb92a48cee/Delt skrivebord/Data Science/Speciale/Energinet/Delte scripts/Speciale_Kode/Shallow learners/SVR2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="8_{D4943CA0-FA4F-4FC1-A64B-712AE16DD25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1D7653F-6225-4609-AC09-0FDC148D692D}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="8_{D4943CA0-FA4F-4FC1-A64B-712AE16DD25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{094A97A5-9722-4552-91F2-B6F15755745C}"/>
   <bookViews>
-    <workbookView xWindow="1770" yWindow="30" windowWidth="25860" windowHeight="15450" xr2:uid="{3563A2C9-D8E3-4CA6-B000-C9444678AE5F}"/>
+    <workbookView xWindow="390" yWindow="30" windowWidth="26355" windowHeight="15450" xr2:uid="{3563A2C9-D8E3-4CA6-B000-C9444678AE5F}"/>
   </bookViews>
   <sheets>
     <sheet name="DK1_hyperparameter_results" sheetId="2" r:id="rId1"/>
@@ -134,9 +134,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -156,10 +155,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -885,13 +880,13 @@
       <c r="C18">
         <v>2</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" t="s">
         <v>8</v>
       </c>
       <c r="E18">
         <v>0.5</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" t="s">
         <v>9</v>
       </c>
       <c r="G18">
@@ -908,13 +903,13 @@
       <c r="C19">
         <v>2</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" t="s">
         <v>8</v>
       </c>
       <c r="E19">
         <v>0.5</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" t="s">
         <v>9</v>
       </c>
       <c r="G19">
@@ -931,13 +926,13 @@
       <c r="C20">
         <v>2</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" t="s">
         <v>8</v>
       </c>
       <c r="E20">
         <v>0.5</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F20" t="s">
         <v>9</v>
       </c>
       <c r="G20">
@@ -954,13 +949,13 @@
       <c r="C21">
         <v>2</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" t="s">
         <v>8</v>
       </c>
       <c r="E21">
         <v>0.05</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F21" t="s">
         <v>9</v>
       </c>
       <c r="G21">
@@ -977,13 +972,13 @@
       <c r="C22">
         <v>2</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" t="s">
         <v>8</v>
       </c>
       <c r="E22">
         <v>0.05</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="F22" t="s">
         <v>9</v>
       </c>
       <c r="G22">
@@ -1000,13 +995,13 @@
       <c r="C23">
         <v>2</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" t="s">
         <v>8</v>
       </c>
       <c r="E23">
         <v>0.05</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="F23" t="s">
         <v>9</v>
       </c>
       <c r="G23">
@@ -1023,13 +1018,13 @@
       <c r="C24">
         <v>2</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" t="s">
         <v>8</v>
       </c>
       <c r="E24">
         <v>0.5</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="F24" t="s">
         <v>9</v>
       </c>
       <c r="G24">
@@ -1046,13 +1041,13 @@
       <c r="C25">
         <v>2</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" t="s">
         <v>8</v>
       </c>
       <c r="E25">
         <v>0.5</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F25" t="s">
         <v>9</v>
       </c>
       <c r="G25">
@@ -1069,13 +1064,13 @@
       <c r="C26">
         <v>2</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" t="s">
         <v>8</v>
       </c>
       <c r="E26">
         <v>0.5</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" t="s">
         <v>9</v>
       </c>
       <c r="G26">
@@ -1092,13 +1087,13 @@
       <c r="C27">
         <v>2</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" t="s">
         <v>8</v>
       </c>
       <c r="E27">
         <v>0.05</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F27" t="s">
         <v>9</v>
       </c>
       <c r="G27">
@@ -1115,13 +1110,13 @@
       <c r="C28">
         <v>2</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" t="s">
         <v>8</v>
       </c>
       <c r="E28">
         <v>0.05</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" t="s">
         <v>9</v>
       </c>
       <c r="G28">
@@ -1138,13 +1133,13 @@
       <c r="C29">
         <v>2</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" t="s">
         <v>8</v>
       </c>
       <c r="E29">
         <v>0.05</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="F29" t="s">
         <v>9</v>
       </c>
       <c r="G29">
@@ -1161,13 +1156,13 @@
       <c r="C30">
         <v>2</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" t="s">
         <v>8</v>
       </c>
       <c r="E30">
         <v>0.5</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="F30" t="s">
         <v>9</v>
       </c>
       <c r="G30">
@@ -1184,13 +1179,13 @@
       <c r="C31">
         <v>2</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D31" t="s">
         <v>8</v>
       </c>
       <c r="E31">
         <v>0.5</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="F31" t="s">
         <v>9</v>
       </c>
       <c r="G31">
@@ -1207,13 +1202,13 @@
       <c r="C32">
         <v>2</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D32" t="s">
         <v>8</v>
       </c>
       <c r="E32">
         <v>0.5</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F32" t="s">
         <v>9</v>
       </c>
       <c r="G32">
@@ -1230,13 +1225,13 @@
       <c r="C33">
         <v>2</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" t="s">
         <v>8</v>
       </c>
       <c r="E33">
         <v>0.05</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="F33" t="s">
         <v>9</v>
       </c>
       <c r="G33">
@@ -1253,13 +1248,13 @@
       <c r="C34">
         <v>2</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="D34" t="s">
         <v>8</v>
       </c>
       <c r="E34">
         <v>0.05</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="F34" t="s">
         <v>9</v>
       </c>
       <c r="G34">
@@ -1276,13 +1271,13 @@
       <c r="C35">
         <v>2</v>
       </c>
-      <c r="D35" s="1" t="s">
+      <c r="D35" t="s">
         <v>8</v>
       </c>
       <c r="E35">
         <v>0.05</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="F35" t="s">
         <v>9</v>
       </c>
       <c r="G35">
@@ -1299,13 +1294,13 @@
       <c r="C36">
         <v>0</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="D36" t="s">
         <v>10</v>
       </c>
       <c r="E36">
         <v>0</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="F36" t="s">
         <v>11</v>
       </c>
       <c r="G36">
@@ -1322,13 +1317,13 @@
       <c r="C37">
         <v>0</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D37" t="s">
         <v>10</v>
       </c>
       <c r="E37">
         <v>0</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="F37" t="s">
         <v>11</v>
       </c>
       <c r="G37">
@@ -1345,13 +1340,13 @@
       <c r="C38">
         <v>0</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D38" t="s">
         <v>10</v>
       </c>
       <c r="E38">
         <v>0</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="F38" t="s">
         <v>11</v>
       </c>
       <c r="G38">
@@ -1368,13 +1363,13 @@
       <c r="C39">
         <v>0</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D39" t="s">
         <v>10</v>
       </c>
       <c r="E39">
         <v>0</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="F39" t="s">
         <v>11</v>
       </c>
       <c r="G39">
@@ -1391,13 +1386,13 @@
       <c r="C40">
         <v>0</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D40" t="s">
         <v>10</v>
       </c>
       <c r="E40">
         <v>0</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="F40" t="s">
         <v>11</v>
       </c>
       <c r="G40">
@@ -1414,13 +1409,13 @@
       <c r="C41">
         <v>0</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D41" t="s">
         <v>10</v>
       </c>
       <c r="E41">
         <v>0</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="F41" t="s">
         <v>11</v>
       </c>
       <c r="G41">
@@ -1437,13 +1432,13 @@
       <c r="C42">
         <v>0</v>
       </c>
-      <c r="D42" s="1" t="s">
+      <c r="D42" t="s">
         <v>8</v>
       </c>
       <c r="E42">
         <v>0</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="F42" t="s">
         <v>11</v>
       </c>
       <c r="G42">
@@ -1460,13 +1455,13 @@
       <c r="C43">
         <v>0</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="D43" t="s">
         <v>8</v>
       </c>
       <c r="E43">
         <v>0</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="F43" t="s">
         <v>11</v>
       </c>
       <c r="G43">
@@ -1483,13 +1478,13 @@
       <c r="C44">
         <v>0</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="D44" t="s">
         <v>8</v>
       </c>
       <c r="E44">
         <v>0</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="F44" t="s">
         <v>11</v>
       </c>
       <c r="G44">
@@ -1506,13 +1501,13 @@
       <c r="C45">
         <v>0</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="D45" t="s">
         <v>12</v>
       </c>
       <c r="E45">
         <v>0</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="F45" t="s">
         <v>11</v>
       </c>
       <c r="G45">
@@ -1529,13 +1524,13 @@
       <c r="C46">
         <v>0</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D46" t="s">
         <v>12</v>
       </c>
       <c r="E46">
         <v>0</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F46" t="s">
         <v>11</v>
       </c>
       <c r="G46">
@@ -1552,13 +1547,13 @@
       <c r="C47">
         <v>0</v>
       </c>
-      <c r="D47" s="1" t="s">
+      <c r="D47" t="s">
         <v>12</v>
       </c>
       <c r="E47">
         <v>0</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="F47" t="s">
         <v>11</v>
       </c>
       <c r="G47">
@@ -1575,13 +1570,13 @@
       <c r="C48">
         <v>0</v>
       </c>
-      <c r="D48" s="1" t="s">
+      <c r="D48" t="s">
         <v>12</v>
       </c>
       <c r="E48">
         <v>0</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="F48" t="s">
         <v>11</v>
       </c>
       <c r="G48">
@@ -1598,13 +1593,13 @@
       <c r="C49">
         <v>0</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="D49" t="s">
         <v>12</v>
       </c>
       <c r="E49">
         <v>0</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="F49" t="s">
         <v>11</v>
       </c>
       <c r="G49">
@@ -1621,13 +1616,13 @@
       <c r="C50">
         <v>0</v>
       </c>
-      <c r="D50" s="1" t="s">
+      <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50">
         <v>0</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="F50" t="s">
         <v>11</v>
       </c>
       <c r="G50">
@@ -1644,13 +1639,13 @@
       <c r="C51">
         <v>0</v>
       </c>
-      <c r="D51" s="1" t="s">
+      <c r="D51" t="s">
         <v>8</v>
       </c>
       <c r="E51">
         <v>0</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="F51" t="s">
         <v>11</v>
       </c>
       <c r="G51">
@@ -1667,13 +1662,13 @@
       <c r="C52">
         <v>0</v>
       </c>
-      <c r="D52" s="1" t="s">
+      <c r="D52" t="s">
         <v>8</v>
       </c>
       <c r="E52">
         <v>0</v>
       </c>
-      <c r="F52" s="1" t="s">
+      <c r="F52" t="s">
         <v>11</v>
       </c>
       <c r="G52">
@@ -1690,13 +1685,13 @@
       <c r="C53">
         <v>0</v>
       </c>
-      <c r="D53" s="1" t="s">
+      <c r="D53" t="s">
         <v>8</v>
       </c>
       <c r="E53">
         <v>0</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="F53" t="s">
         <v>11</v>
       </c>
       <c r="G53">
@@ -1713,13 +1708,13 @@
       <c r="C54">
         <v>0</v>
       </c>
-      <c r="D54" s="1" t="s">
+      <c r="D54" t="s">
         <v>10</v>
       </c>
       <c r="E54">
         <v>0</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="F54" t="s">
         <v>11</v>
       </c>
       <c r="G54">
@@ -1736,13 +1731,13 @@
       <c r="C55">
         <v>0</v>
       </c>
-      <c r="D55" s="1" t="s">
+      <c r="D55" t="s">
         <v>10</v>
       </c>
       <c r="E55">
         <v>0</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="F55" t="s">
         <v>11</v>
       </c>
       <c r="G55">
@@ -1759,13 +1754,13 @@
       <c r="C56">
         <v>0</v>
       </c>
-      <c r="D56" s="1" t="s">
+      <c r="D56" t="s">
         <v>10</v>
       </c>
       <c r="E56">
         <v>0</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="F56" t="s">
         <v>11</v>
       </c>
       <c r="G56">
@@ -1782,13 +1777,13 @@
       <c r="C57">
         <v>0</v>
       </c>
-      <c r="D57" s="1" t="s">
+      <c r="D57" t="s">
         <v>12</v>
       </c>
       <c r="E57">
         <v>0</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="F57" t="s">
         <v>11</v>
       </c>
       <c r="G57">
@@ -1805,13 +1800,13 @@
       <c r="C58">
         <v>0</v>
       </c>
-      <c r="D58" s="1" t="s">
+      <c r="D58" t="s">
         <v>12</v>
       </c>
       <c r="E58">
         <v>0</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="F58" t="s">
         <v>11</v>
       </c>
       <c r="G58">
@@ -1828,13 +1823,13 @@
       <c r="C59">
         <v>0</v>
       </c>
-      <c r="D59" s="1" t="s">
+      <c r="D59" t="s">
         <v>12</v>
       </c>
       <c r="E59">
         <v>0</v>
       </c>
-      <c r="F59" s="1" t="s">
+      <c r="F59" t="s">
         <v>11</v>
       </c>
       <c r="G59">
@@ -1851,13 +1846,13 @@
       <c r="C60">
         <v>0</v>
       </c>
-      <c r="D60" s="1" t="s">
+      <c r="D60" t="s">
         <v>8</v>
       </c>
       <c r="E60">
         <v>0</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="F60" t="s">
         <v>11</v>
       </c>
       <c r="G60">
@@ -1874,13 +1869,13 @@
       <c r="C61">
         <v>0</v>
       </c>
-      <c r="D61" s="1" t="s">
+      <c r="D61" t="s">
         <v>8</v>
       </c>
       <c r="E61">
         <v>0</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="F61" t="s">
         <v>11</v>
       </c>
       <c r="G61">
@@ -1897,13 +1892,13 @@
       <c r="C62">
         <v>0</v>
       </c>
-      <c r="D62" s="1" t="s">
+      <c r="D62" t="s">
         <v>8</v>
       </c>
       <c r="E62">
         <v>0</v>
       </c>
-      <c r="F62" s="1" t="s">
+      <c r="F62" t="s">
         <v>11</v>
       </c>
       <c r="G62">

</xml_diff>